<commit_message>
Student import via excel
</commit_message>
<xml_diff>
--- a/old/src/main/webapp/resources/students.xlsx
+++ b/old/src/main/webapp/resources/students.xlsx
@@ -1,25 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="989"/>
+    <workbookView windowWidth="28695" windowHeight="13650" tabRatio="989"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37">
   <si>
     <t>FORM 1 N</t>
   </si>
@@ -54,43 +49,43 @@
     <t>Day</t>
   </si>
   <si>
+    <t>Dynah</t>
+  </si>
+  <si>
+    <t>Mwende</t>
+  </si>
+  <si>
     <t>F</t>
   </si>
   <si>
+    <t>Marry</t>
+  </si>
+  <si>
+    <t>Akoth</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>Doris</t>
+  </si>
+  <si>
+    <t>Nd'ung'u</t>
+  </si>
+  <si>
+    <t>Obed</t>
+  </si>
+  <si>
+    <t>Muthomi</t>
+  </si>
+  <si>
+    <t>Newton</t>
+  </si>
+  <si>
+    <t>Muthengi</t>
+  </si>
+  <si>
     <t>Boarder</t>
-  </si>
-  <si>
-    <t>Marry</t>
-  </si>
-  <si>
-    <t>Akoth</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>Doris</t>
-  </si>
-  <si>
-    <t>Nd'ung'u</t>
-  </si>
-  <si>
-    <t>Dynah</t>
-  </si>
-  <si>
-    <t>Mwende</t>
-  </si>
-  <si>
-    <t>Obed</t>
-  </si>
-  <si>
-    <t>Muthomi</t>
-  </si>
-  <si>
-    <t>Newton</t>
-  </si>
-  <si>
-    <t>Muthengi</t>
   </si>
   <si>
     <t>Regina</t>
@@ -135,24 +130,366 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -160,27 +497,308 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
+    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
+    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
+    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
+    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
+    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
+    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
+    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
+    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
+    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
+    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
+    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
+    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
+    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
+    <cellStyle name="Accent1" xfId="19" builtinId="29"/>
+    <cellStyle name="Comma[0]" xfId="20" builtinId="6"/>
+    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
+    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
+    <cellStyle name="Total" xfId="25" builtinId="25"/>
+    <cellStyle name="Output" xfId="26" builtinId="21"/>
+    <cellStyle name="Currency" xfId="27" builtinId="4"/>
+    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
+    <cellStyle name="Note" xfId="29" builtinId="10"/>
+    <cellStyle name="Input" xfId="30" builtinId="20"/>
+    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
+    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
+    <cellStyle name="Good" xfId="33" builtinId="26"/>
+    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
+    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Currency[0]" xfId="37" builtinId="7"/>
+    <cellStyle name="Heading 1" xfId="38" builtinId="16"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50"/>
+    <cellStyle name="Title" xfId="40" builtinId="15"/>
+    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
+    <cellStyle name="20% - Accent1" xfId="42" builtinId="30"/>
+    <cellStyle name="Hyperlink" xfId="43" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="44" builtinId="9"/>
+    <cellStyle name="Heading 2" xfId="45" builtinId="17"/>
+    <cellStyle name="Comma" xfId="46" builtinId="3"/>
+    <cellStyle name="Check Cell" xfId="47" builtinId="23"/>
+    <cellStyle name="Percent" xfId="48" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2"/>
 </styleSheet>
 </file>
 
@@ -189,10 +807,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText" lastClr="212121"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window" lastClr="F3F3F3"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -227,7 +845,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -262,7 +880,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -437,32 +1055,28 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr/>
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="11.5703125"/>
-    <col min="2" max="2" width="15.140625"/>
+    <col min="1" max="1" width="11.5666666666667"/>
+    <col min="2" max="2" width="15.1416666666667"/>
     <col min="3" max="3" width="15"/>
     <col min="4" max="4" width="16"/>
-    <col min="5" max="1025" width="11.5703125"/>
+    <col min="5" max="1025" width="11.5666666666667"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -482,7 +1096,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>100</v>
       </c>
@@ -502,18 +1116,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>101</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>389</v>
@@ -522,18 +1136,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>234</v>
@@ -542,18 +1156,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>103</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
         <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
       </c>
       <c r="E6">
         <v>306</v>
@@ -562,15 +1176,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>104</v>
       </c>
       <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -582,15 +1196,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>105</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
         <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
@@ -599,10 +1213,10 @@
         <v>286</v>
       </c>
       <c r="F8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>106</v>
       </c>
@@ -613,16 +1227,16 @@
         <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>312</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>107</v>
       </c>
@@ -639,10 +1253,10 @@
         <v>299</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>108</v>
       </c>
@@ -653,16 +1267,16 @@
         <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E11">
         <v>401</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>109</v>
       </c>
@@ -670,7 +1284,7 @@
         <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
         <v>9</v>
@@ -679,10 +1293,10 @@
         <v>234</v>
       </c>
       <c r="F12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>110</v>
       </c>
@@ -699,10 +1313,10 @@
         <v>306</v>
       </c>
       <c r="F13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>111</v>
       </c>
@@ -719,10 +1333,10 @@
         <v>300</v>
       </c>
       <c r="F14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>112</v>
       </c>
@@ -739,12 +1353,18 @@
         <v>286</v>
       </c>
       <c r="F15" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="0" scale="0" orientation="portrait" usePrinterDefaults="0" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0" copies="0"/>
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E$1:E$1048576">
+      <formula1>100</formula1>
+      <formula2>500</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7875" right="0.7875" top="1.02430555555556" bottom="1.02430555555556" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>

</xml_diff>